<commit_message>
BIG new ms_endemism -> ms_suit; ms_merge = ms_suit * ms_er
</commit_message>
<xml_diff>
--- a/figs/msens-summary_programareas_v3/table_programarea_scores_v3.xlsx
+++ b/figs/msens-summary_programareas_v3/table_programarea_scores_v3.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">Program Area</t>
   </si>
@@ -23,21 +23,9 @@
     <t xml:space="preserve">Primary Production</t>
   </si>
   <si>
-    <t xml:space="preserve">Bird</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coral</t>
-  </si>
-  <si>
     <t xml:space="preserve">Fish</t>
   </si>
   <si>
-    <t xml:space="preserve">Invertebrate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mammal</t>
-  </si>
-  <si>
     <t xml:space="preserve">Other</t>
   </si>
   <si>
@@ -47,45 +35,48 @@
     <t xml:space="preserve">Hope Basin (HOP)</t>
   </si>
   <si>
+    <t xml:space="preserve">Chukchi Sea (CHU)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cook Inlet (COK)</t>
   </si>
   <si>
     <t xml:space="preserve">GOA Program Area A (GAA)</t>
   </si>
   <si>
+    <t xml:space="preserve">Gulf of Alaska (GOA)</t>
+  </si>
+  <si>
     <t xml:space="preserve">St. George Basin (GEO)</t>
   </si>
   <si>
-    <t xml:space="preserve">Gulf of Alaska (GOA)</t>
+    <t xml:space="preserve">Aleutian Arc (ALA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kodiak (KOD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOA Program Area B (GAB)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Norton Basin (NOR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shumagin (SHU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beaufort Sea (BFT)</t>
   </si>
   <si>
     <t xml:space="preserve">Southern California (SOC)</t>
   </si>
   <si>
-    <t xml:space="preserve">Chukchi Sea (CHU)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOA Program Area B (GAB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Norton Basin (NOR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kodiak (KOD)</t>
+    <t xml:space="preserve">St. Matthew-Hall (MAT)</t>
   </si>
   <si>
     <t xml:space="preserve">Navarin Basin (NAV)</t>
   </si>
   <si>
-    <t xml:space="preserve">Aleutian Arc (ALA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shumagin (SHU)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">St. Matthew-Hall (MAT)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Central California (CEC)</t>
   </si>
   <si>
@@ -95,13 +86,10 @@
     <t xml:space="preserve">Bowers Basin (BOW)</t>
   </si>
   <si>
-    <t xml:space="preserve">Beaufort Sea (BFT)</t>
+    <t xml:space="preserve">High Arctic (HAR)</t>
   </si>
   <si>
     <t xml:space="preserve">Aleutian Basin (ALB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High Arctic (HAR)</t>
   </si>
 </sst>
 </file>
@@ -449,657 +437,405 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="C2" t="n">
         <v>27</v>
       </c>
       <c r="D2" t="n">
-        <v>49</v>
+        <v>87</v>
       </c>
       <c r="E2" t="n">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="F2" t="n">
-        <v>70</v>
-      </c>
-      <c r="G2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H2" t="n">
-        <v>83</v>
-      </c>
-      <c r="I2" t="n">
-        <v>33</v>
-      </c>
-      <c r="J2" t="n">
         <v>52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C3" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="D3" t="n">
-        <v>94</v>
+        <v>54</v>
       </c>
       <c r="E3" t="n">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="F3" t="n">
-        <v>70</v>
-      </c>
-      <c r="G3" t="n">
-        <v>44</v>
-      </c>
-      <c r="H3" t="n">
-        <v>67</v>
-      </c>
-      <c r="I3" t="n">
-        <v>41</v>
-      </c>
-      <c r="J3" t="n">
-        <v>22</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="D4" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="F4" t="n">
-        <v>31</v>
-      </c>
-      <c r="G4" t="n">
-        <v>32</v>
-      </c>
-      <c r="H4" t="n">
-        <v>45</v>
-      </c>
-      <c r="I4" t="n">
-        <v>26</v>
-      </c>
-      <c r="J4" t="n">
-        <v>382</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B5" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D5" t="n">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="E5" t="n">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="F5" t="n">
-        <v>37</v>
-      </c>
-      <c r="G5" t="n">
-        <v>32</v>
-      </c>
-      <c r="H5" t="n">
-        <v>73</v>
-      </c>
-      <c r="I5" t="n">
-        <v>31</v>
-      </c>
-      <c r="J5" t="n">
-        <v>283</v>
+        <v>382</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B6" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C6" t="n">
         <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="E6" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="F6" t="n">
-        <v>28</v>
-      </c>
-      <c r="G6" t="n">
-        <v>27</v>
-      </c>
-      <c r="H6" t="n">
-        <v>65</v>
-      </c>
-      <c r="I6" t="n">
-        <v>23</v>
-      </c>
-      <c r="J6" t="n">
         <v>383</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B7" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C7" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>57</v>
+        <v>32</v>
       </c>
       <c r="E7" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="F7" t="n">
-        <v>24</v>
-      </c>
-      <c r="G7" t="n">
-        <v>18</v>
-      </c>
-      <c r="H7" t="n">
-        <v>68</v>
-      </c>
-      <c r="I7" t="n">
-        <v>15</v>
-      </c>
-      <c r="J7" t="n">
-        <v>276</v>
+        <v>283</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B8" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="E8" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F8" t="n">
-        <v>17</v>
-      </c>
-      <c r="G8" t="n">
-        <v>46</v>
-      </c>
-      <c r="H8" t="n">
-        <v>47</v>
-      </c>
-      <c r="I8" t="n">
-        <v>34</v>
-      </c>
-      <c r="J8" t="n">
-        <v>252</v>
+        <v>870</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B9" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D9" t="n">
-        <v>82</v>
+        <v>25</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="F9" t="n">
-        <v>14</v>
-      </c>
-      <c r="G9" t="n">
-        <v>12</v>
-      </c>
-      <c r="H9" t="n">
-        <v>60</v>
-      </c>
-      <c r="I9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J9" t="n">
-        <v>82</v>
+        <v>274</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B10" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C10" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>66</v>
+        <v>17</v>
       </c>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F10" t="n">
-        <v>12</v>
-      </c>
-      <c r="G10" t="n">
-        <v>12</v>
-      </c>
-      <c r="H10" t="n">
-        <v>50</v>
-      </c>
-      <c r="I10" t="n">
-        <v>7</v>
-      </c>
-      <c r="J10" t="n">
-        <v>98</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B11" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D11" t="n">
-        <v>46</v>
+        <v>5</v>
       </c>
       <c r="E11" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F11" t="n">
-        <v>26</v>
-      </c>
-      <c r="G11" t="n">
-        <v>19</v>
-      </c>
-      <c r="H11" t="n">
-        <v>49</v>
-      </c>
-      <c r="I11" t="n">
-        <v>17</v>
-      </c>
-      <c r="J11" t="n">
-        <v>274</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B12" t="n">
+        <v>21</v>
+      </c>
+      <c r="C12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" t="n">
         <v>24</v>
       </c>
-      <c r="C12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D12" t="n">
-        <v>36</v>
-      </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F12" t="n">
-        <v>20</v>
-      </c>
-      <c r="G12" t="n">
-        <v>14</v>
-      </c>
-      <c r="H12" t="n">
-        <v>67</v>
-      </c>
-      <c r="I12" t="n">
-        <v>17</v>
-      </c>
-      <c r="J12" t="n">
-        <v>137</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B13" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D13" t="n">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="E13" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F13" t="n">
-        <v>22</v>
-      </c>
-      <c r="G13" t="n">
-        <v>15</v>
-      </c>
-      <c r="H13" t="n">
-        <v>45</v>
-      </c>
-      <c r="I13" t="n">
-        <v>18</v>
-      </c>
-      <c r="J13" t="n">
-        <v>870</v>
+        <v>262</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B14" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D14" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="E14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F14" t="n">
-        <v>27</v>
-      </c>
-      <c r="G14" t="n">
-        <v>17</v>
-      </c>
-      <c r="H14" t="n">
-        <v>44</v>
-      </c>
-      <c r="I14" t="n">
-        <v>16</v>
-      </c>
-      <c r="J14" t="n">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B15" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C15" t="n">
         <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="E15" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="F15" t="n">
-        <v>11</v>
-      </c>
-      <c r="G15" t="n">
-        <v>12</v>
-      </c>
-      <c r="H15" t="n">
-        <v>44</v>
-      </c>
-      <c r="I15" t="n">
-        <v>8</v>
-      </c>
-      <c r="J15" t="n">
         <v>220</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B16" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C16" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="F16" t="n">
-        <v>12</v>
-      </c>
-      <c r="G16" t="n">
-        <v>7</v>
-      </c>
-      <c r="H16" t="n">
-        <v>59</v>
-      </c>
-      <c r="I16" t="n">
-        <v>5</v>
-      </c>
-      <c r="J16" t="n">
-        <v>144</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B17" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C17" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D17" t="n">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F17" t="n">
-        <v>11</v>
-      </c>
-      <c r="G17" t="n">
-        <v>8</v>
-      </c>
-      <c r="H17" t="n">
-        <v>65</v>
-      </c>
-      <c r="I17" t="n">
-        <v>8</v>
-      </c>
-      <c r="J17" t="n">
-        <v>171</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B18" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D18" t="n">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E18" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F18" t="n">
-        <v>9</v>
-      </c>
-      <c r="G18" t="n">
-        <v>6</v>
-      </c>
-      <c r="H18" t="n">
-        <v>59</v>
-      </c>
-      <c r="I18" t="n">
-        <v>10</v>
-      </c>
-      <c r="J18" t="n">
-        <v>353</v>
+        <v>171</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B19" t="n">
+        <v>12</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>20</v>
+      </c>
+      <c r="E19" t="n">
         <v>13</v>
       </c>
-      <c r="C19" t="n">
-        <v>5</v>
-      </c>
-      <c r="D19" t="n">
-        <v>8</v>
-      </c>
-      <c r="E19" t="n">
-        <v>17</v>
-      </c>
       <c r="F19" t="n">
-        <v>4</v>
-      </c>
-      <c r="G19" t="n">
-        <v>18</v>
-      </c>
-      <c r="H19" t="n">
-        <v>20</v>
-      </c>
-      <c r="I19" t="n">
-        <v>21</v>
-      </c>
-      <c r="J19" t="n">
-        <v>262</v>
+        <v>353</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B20" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D20" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E20" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="F20" t="n">
-        <v>3</v>
-      </c>
-      <c r="G20" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" t="n">
-        <v>54</v>
-      </c>
-      <c r="I20" t="n">
-        <v>5</v>
-      </c>
-      <c r="J20" t="n">
-        <v>167</v>
+        <v>438</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B21" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C21" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E21" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="F21" t="n">
-        <v>6</v>
-      </c>
-      <c r="G21" t="n">
-        <v>16</v>
-      </c>
-      <c r="H21" t="n">
-        <v>2</v>
-      </c>
-      <c r="I21" t="n">
-        <v>23</v>
-      </c>
-      <c r="J21" t="n">
-        <v>438</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "BIG new ms_endemism -> ms_suit; ms_merge = ms_suit * ms_er"
This reverts commit 6c3e49c0750f8873529674fa57fde05cd14ed3d4.
</commit_message>
<xml_diff>
--- a/figs/msens-summary_programareas_v3/table_programarea_scores_v3.xlsx
+++ b/figs/msens-summary_programareas_v3/table_programarea_scores_v3.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t xml:space="preserve">Program Area</t>
   </si>
@@ -23,9 +23,21 @@
     <t xml:space="preserve">Primary Production</t>
   </si>
   <si>
+    <t xml:space="preserve">Bird</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coral</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fish</t>
   </si>
   <si>
+    <t xml:space="preserve">Invertebrate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mammal</t>
+  </si>
+  <si>
     <t xml:space="preserve">Other</t>
   </si>
   <si>
@@ -35,61 +47,61 @@
     <t xml:space="preserve">Hope Basin (HOP)</t>
   </si>
   <si>
+    <t xml:space="preserve">Cook Inlet (COK)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOA Program Area A (GAA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">St. George Basin (GEO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gulf of Alaska (GOA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Southern California (SOC)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chukchi Sea (CHU)</t>
   </si>
   <si>
-    <t xml:space="preserve">Cook Inlet (COK)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOA Program Area A (GAA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gulf of Alaska (GOA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">St. George Basin (GEO)</t>
+    <t xml:space="preserve">GOA Program Area B (GAB)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Norton Basin (NOR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kodiak (KOD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Navarin Basin (NAV)</t>
   </si>
   <si>
     <t xml:space="preserve">Aleutian Arc (ALA)</t>
   </si>
   <si>
-    <t xml:space="preserve">Kodiak (KOD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOA Program Area B (GAB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Norton Basin (NOR)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Shumagin (SHU)</t>
   </si>
   <si>
+    <t xml:space="preserve">St. Matthew-Hall (MAT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Central California (CEC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Northern California (NOC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bowers Basin (BOW)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Beaufort Sea (BFT)</t>
   </si>
   <si>
-    <t xml:space="preserve">Southern California (SOC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">St. Matthew-Hall (MAT)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Navarin Basin (NAV)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Central California (CEC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Northern California (NOC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bowers Basin (BOW)</t>
+    <t xml:space="preserve">Aleutian Basin (ALB)</t>
   </si>
   <si>
     <t xml:space="preserve">High Arctic (HAR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aleutian Basin (ALB)</t>
   </si>
 </sst>
 </file>
@@ -437,405 +449,657 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="C2" t="n">
         <v>27</v>
       </c>
       <c r="D2" t="n">
-        <v>87</v>
+        <v>49</v>
       </c>
       <c r="E2" t="n">
+        <v>48</v>
+      </c>
+      <c r="F2" t="n">
+        <v>70</v>
+      </c>
+      <c r="G2" t="n">
         <v>68</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
+        <v>83</v>
+      </c>
+      <c r="I2" t="n">
+        <v>33</v>
+      </c>
+      <c r="J2" t="n">
         <v>52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C3" t="n">
+        <v>21</v>
+      </c>
+      <c r="D3" t="n">
+        <v>94</v>
+      </c>
+      <c r="E3" t="n">
+        <v>28</v>
+      </c>
+      <c r="F3" t="n">
+        <v>70</v>
+      </c>
+      <c r="G3" t="n">
         <v>44</v>
       </c>
-      <c r="C3" t="n">
-        <v>7</v>
-      </c>
-      <c r="D3" t="n">
-        <v>54</v>
-      </c>
-      <c r="E3" t="n">
-        <v>53</v>
-      </c>
-      <c r="F3" t="n">
-        <v>252</v>
+      <c r="H3" t="n">
+        <v>67</v>
+      </c>
+      <c r="I3" t="n">
+        <v>41</v>
+      </c>
+      <c r="J3" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B4" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C4" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E4" t="n">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>22</v>
+        <v>31</v>
+      </c>
+      <c r="G4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H4" t="n">
+        <v>45</v>
+      </c>
+      <c r="I4" t="n">
+        <v>26</v>
+      </c>
+      <c r="J4" t="n">
+        <v>382</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B5" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C5" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
+        <v>49</v>
+      </c>
+      <c r="E5" t="n">
+        <v>27</v>
+      </c>
+      <c r="F5" t="n">
         <v>37</v>
       </c>
-      <c r="E5" t="n">
-        <v>41</v>
-      </c>
-      <c r="F5" t="n">
-        <v>382</v>
+      <c r="G5" t="n">
+        <v>32</v>
+      </c>
+      <c r="H5" t="n">
+        <v>73</v>
+      </c>
+      <c r="I5" t="n">
+        <v>31</v>
+      </c>
+      <c r="J5" t="n">
+        <v>283</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" t="n">
         <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="E6" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="F6" t="n">
+        <v>28</v>
+      </c>
+      <c r="G6" t="n">
+        <v>27</v>
+      </c>
+      <c r="H6" t="n">
+        <v>65</v>
+      </c>
+      <c r="I6" t="n">
+        <v>23</v>
+      </c>
+      <c r="J6" t="n">
         <v>383</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B7" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D7" t="n">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="E7" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="F7" t="n">
-        <v>283</v>
+        <v>24</v>
+      </c>
+      <c r="G7" t="n">
+        <v>18</v>
+      </c>
+      <c r="H7" t="n">
+        <v>68</v>
+      </c>
+      <c r="I7" t="n">
+        <v>15</v>
+      </c>
+      <c r="J7" t="n">
+        <v>276</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" t="n">
+        <v>15</v>
+      </c>
+      <c r="F8" t="n">
+        <v>17</v>
+      </c>
+      <c r="G8" t="n">
+        <v>46</v>
+      </c>
+      <c r="H8" t="n">
+        <v>47</v>
+      </c>
+      <c r="I8" t="n">
         <v>34</v>
       </c>
-      <c r="E8" t="n">
-        <v>23</v>
-      </c>
-      <c r="F8" t="n">
-        <v>870</v>
+      <c r="J8" t="n">
+        <v>252</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B9" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C9" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>25</v>
+        <v>82</v>
       </c>
       <c r="E9" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>274</v>
+        <v>14</v>
+      </c>
+      <c r="G9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H9" t="n">
+        <v>60</v>
+      </c>
+      <c r="I9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J9" t="n">
+        <v>82</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B10" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D10" t="n">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="E10" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F10" t="n">
-        <v>82</v>
+        <v>12</v>
+      </c>
+      <c r="G10" t="n">
+        <v>12</v>
+      </c>
+      <c r="H10" t="n">
+        <v>50</v>
+      </c>
+      <c r="I10" t="n">
+        <v>7</v>
+      </c>
+      <c r="J10" t="n">
+        <v>98</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B11" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C11" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="E11" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F11" t="n">
-        <v>98</v>
+        <v>26</v>
+      </c>
+      <c r="G11" t="n">
+        <v>19</v>
+      </c>
+      <c r="H11" t="n">
+        <v>49</v>
+      </c>
+      <c r="I11" t="n">
+        <v>17</v>
+      </c>
+      <c r="J11" t="n">
+        <v>274</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B12" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="E12" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="F12" t="n">
-        <v>278</v>
+        <v>20</v>
+      </c>
+      <c r="G12" t="n">
+        <v>14</v>
+      </c>
+      <c r="H12" t="n">
+        <v>67</v>
+      </c>
+      <c r="I12" t="n">
+        <v>17</v>
+      </c>
+      <c r="J12" t="n">
+        <v>137</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B13" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C13" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="E13" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="F13" t="n">
-        <v>262</v>
+        <v>22</v>
+      </c>
+      <c r="G13" t="n">
+        <v>15</v>
+      </c>
+      <c r="H13" t="n">
+        <v>45</v>
+      </c>
+      <c r="I13" t="n">
+        <v>18</v>
+      </c>
+      <c r="J13" t="n">
+        <v>870</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B14" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C14" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D14" t="n">
+        <v>36</v>
+      </c>
+      <c r="E14" t="n">
+        <v>12</v>
+      </c>
+      <c r="F14" t="n">
         <v>27</v>
       </c>
-      <c r="E14" t="n">
-        <v>20</v>
-      </c>
-      <c r="F14" t="n">
-        <v>276</v>
+      <c r="G14" t="n">
+        <v>17</v>
+      </c>
+      <c r="H14" t="n">
+        <v>44</v>
+      </c>
+      <c r="I14" t="n">
+        <v>16</v>
+      </c>
+      <c r="J14" t="n">
+        <v>278</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B15" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C15" t="n">
         <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>7</v>
+        <v>57</v>
       </c>
       <c r="E15" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="F15" t="n">
+        <v>11</v>
+      </c>
+      <c r="G15" t="n">
+        <v>12</v>
+      </c>
+      <c r="H15" t="n">
+        <v>44</v>
+      </c>
+      <c r="I15" t="n">
+        <v>8</v>
+      </c>
+      <c r="J15" t="n">
         <v>220</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" t="n">
         <v>20</v>
       </c>
-      <c r="B16" t="n">
-        <v>16</v>
-      </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E16" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="F16" t="n">
-        <v>137</v>
+        <v>12</v>
+      </c>
+      <c r="G16" t="n">
+        <v>7</v>
+      </c>
+      <c r="H16" t="n">
+        <v>59</v>
+      </c>
+      <c r="I16" t="n">
+        <v>5</v>
+      </c>
+      <c r="J16" t="n">
+        <v>144</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B17" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C17" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D17" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="E17" t="n">
+        <v>8</v>
+      </c>
+      <c r="F17" t="n">
         <v>11</v>
       </c>
-      <c r="F17" t="n">
-        <v>144</v>
+      <c r="G17" t="n">
+        <v>8</v>
+      </c>
+      <c r="H17" t="n">
+        <v>65</v>
+      </c>
+      <c r="I17" t="n">
+        <v>8</v>
+      </c>
+      <c r="J17" t="n">
+        <v>171</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B18" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C18" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="E18" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F18" t="n">
-        <v>171</v>
+        <v>9</v>
+      </c>
+      <c r="G18" t="n">
+        <v>6</v>
+      </c>
+      <c r="H18" t="n">
+        <v>59</v>
+      </c>
+      <c r="I18" t="n">
+        <v>10</v>
+      </c>
+      <c r="J18" t="n">
+        <v>353</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D19" t="n">
+        <v>8</v>
+      </c>
+      <c r="E19" t="n">
+        <v>17</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4</v>
+      </c>
+      <c r="G19" t="n">
+        <v>18</v>
+      </c>
+      <c r="H19" t="n">
         <v>20</v>
       </c>
-      <c r="E19" t="n">
-        <v>13</v>
-      </c>
-      <c r="F19" t="n">
-        <v>353</v>
+      <c r="I19" t="n">
+        <v>21</v>
+      </c>
+      <c r="J19" t="n">
+        <v>262</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B20" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>15</v>
+      </c>
+      <c r="E20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F20" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="n">
+        <v>54</v>
+      </c>
+      <c r="I20" t="n">
         <v>5</v>
       </c>
-      <c r="D20" t="n">
-        <v>11</v>
-      </c>
-      <c r="E20" t="n">
-        <v>22</v>
-      </c>
-      <c r="F20" t="n">
-        <v>438</v>
+      <c r="J20" t="n">
+        <v>167</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B21" t="n">
+        <v>11</v>
+      </c>
+      <c r="C21" t="n">
+        <v>5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>4</v>
+      </c>
+      <c r="E21" t="n">
+        <v>21</v>
+      </c>
+      <c r="F21" t="n">
         <v>6</v>
       </c>
-      <c r="C21" t="n">
+      <c r="G21" t="n">
+        <v>16</v>
+      </c>
+      <c r="H21" t="n">
         <v>2</v>
       </c>
-      <c r="D21" t="n">
-        <v>6</v>
-      </c>
-      <c r="E21" t="n">
-        <v>6</v>
-      </c>
-      <c r="F21" t="n">
-        <v>167</v>
+      <c r="I21" t="n">
+        <v>23</v>
+      </c>
+      <c r="J21" t="n">
+        <v>438</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
quarto render calc_scores, msens-summary_programareas, render_derived_products.qmd
</commit_message>
<xml_diff>
--- a/figs/msens-summary_programareas_v3/table_programarea_scores_v3.xlsx
+++ b/figs/msens-summary_programareas_v3/table_programarea_scores_v3.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">Program Area</t>
   </si>
@@ -23,21 +23,9 @@
     <t xml:space="preserve">Primary Production</t>
   </si>
   <si>
-    <t xml:space="preserve">Bird</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coral</t>
-  </si>
-  <si>
     <t xml:space="preserve">Fish</t>
   </si>
   <si>
-    <t xml:space="preserve">Invertebrate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mammal</t>
-  </si>
-  <si>
     <t xml:space="preserve">Other</t>
   </si>
   <si>
@@ -50,55 +38,55 @@
     <t xml:space="preserve">Cook Inlet (COK)</t>
   </si>
   <si>
+    <t xml:space="preserve">Gulf of Alaska (GOA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">St. George Basin (GEO)</t>
+  </si>
+  <si>
     <t xml:space="preserve">GOA Program Area A (GAA)</t>
   </si>
   <si>
-    <t xml:space="preserve">St. George Basin (GEO)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gulf of Alaska (GOA)</t>
+    <t xml:space="preserve">Kodiak (KOD)</t>
   </si>
   <si>
     <t xml:space="preserve">Southern California (SOC)</t>
   </si>
   <si>
+    <t xml:space="preserve">Norton Basin (NOR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shumagin (SHU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aleutian Arc (ALA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Navarin Basin (NAV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOA Program Area B (GAB)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chukchi Sea (CHU)</t>
   </si>
   <si>
-    <t xml:space="preserve">GOA Program Area B (GAB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Norton Basin (NOR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kodiak (KOD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Navarin Basin (NAV)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aleutian Arc (ALA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shumagin (SHU)</t>
+    <t xml:space="preserve">Central California (CEC)</t>
   </si>
   <si>
     <t xml:space="preserve">St. Matthew-Hall (MAT)</t>
   </si>
   <si>
-    <t xml:space="preserve">Central California (CEC)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Northern California (NOC)</t>
   </si>
   <si>
     <t xml:space="preserve">Bowers Basin (BOW)</t>
   </si>
   <si>
+    <t xml:space="preserve">Aleutian Basin (ALB)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Beaufort Sea (BFT)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aleutian Basin (ALB)</t>
   </si>
   <si>
     <t xml:space="preserve">High Arctic (HAR)</t>
@@ -449,630 +437,390 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C2" t="n">
         <v>27</v>
       </c>
       <c r="D2" t="n">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="E2" t="n">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="F2" t="n">
-        <v>70</v>
-      </c>
-      <c r="G2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H2" t="n">
-        <v>83</v>
-      </c>
-      <c r="I2" t="n">
-        <v>33</v>
-      </c>
-      <c r="J2" t="n">
         <v>52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C3" t="n">
         <v>21</v>
       </c>
       <c r="D3" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="E3" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="F3" t="n">
-        <v>70</v>
-      </c>
-      <c r="G3" t="n">
-        <v>44</v>
-      </c>
-      <c r="H3" t="n">
-        <v>67</v>
-      </c>
-      <c r="I3" t="n">
-        <v>41</v>
-      </c>
-      <c r="J3" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D4" t="n">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F4" t="n">
-        <v>31</v>
-      </c>
-      <c r="G4" t="n">
-        <v>32</v>
-      </c>
-      <c r="H4" t="n">
-        <v>45</v>
-      </c>
-      <c r="I4" t="n">
-        <v>26</v>
-      </c>
-      <c r="J4" t="n">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B5" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C5" t="n">
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="E5" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F5" t="n">
-        <v>37</v>
-      </c>
-      <c r="G5" t="n">
-        <v>32</v>
-      </c>
-      <c r="H5" t="n">
-        <v>73</v>
-      </c>
-      <c r="I5" t="n">
-        <v>31</v>
-      </c>
-      <c r="J5" t="n">
         <v>283</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B6" t="n">
+        <v>33</v>
+      </c>
+      <c r="C6" t="n">
+        <v>11</v>
+      </c>
+      <c r="D6" t="n">
         <v>31</v>
       </c>
-      <c r="C6" t="n">
-        <v>10</v>
-      </c>
-      <c r="D6" t="n">
-        <v>49</v>
-      </c>
       <c r="E6" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F6" t="n">
-        <v>28</v>
-      </c>
-      <c r="G6" t="n">
-        <v>27</v>
-      </c>
-      <c r="H6" t="n">
-        <v>65</v>
-      </c>
-      <c r="I6" t="n">
-        <v>23</v>
-      </c>
-      <c r="J6" t="n">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B7" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C7" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D7" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="E7" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F7" t="n">
-        <v>24</v>
-      </c>
-      <c r="G7" t="n">
-        <v>18</v>
-      </c>
-      <c r="H7" t="n">
-        <v>68</v>
-      </c>
-      <c r="I7" t="n">
-        <v>15</v>
-      </c>
-      <c r="J7" t="n">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B8" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C8" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D8" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="E8" t="n">
         <v>15</v>
       </c>
       <c r="F8" t="n">
-        <v>17</v>
-      </c>
-      <c r="G8" t="n">
-        <v>46</v>
-      </c>
-      <c r="H8" t="n">
-        <v>47</v>
-      </c>
-      <c r="I8" t="n">
-        <v>34</v>
-      </c>
-      <c r="J8" t="n">
-        <v>252</v>
+        <v>276</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B9" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D9" t="n">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F9" t="n">
-        <v>14</v>
-      </c>
-      <c r="G9" t="n">
-        <v>12</v>
-      </c>
-      <c r="H9" t="n">
-        <v>60</v>
-      </c>
-      <c r="I9" t="n">
-        <v>6</v>
-      </c>
-      <c r="J9" t="n">
-        <v>82</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B10" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C10" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D10" t="n">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="F10" t="n">
-        <v>12</v>
-      </c>
-      <c r="G10" t="n">
-        <v>12</v>
-      </c>
-      <c r="H10" t="n">
-        <v>50</v>
-      </c>
-      <c r="I10" t="n">
-        <v>7</v>
-      </c>
-      <c r="J10" t="n">
-        <v>98</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B11" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E11" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F11" t="n">
-        <v>26</v>
-      </c>
-      <c r="G11" t="n">
-        <v>19</v>
-      </c>
-      <c r="H11" t="n">
-        <v>49</v>
-      </c>
-      <c r="I11" t="n">
-        <v>17</v>
-      </c>
-      <c r="J11" t="n">
-        <v>274</v>
+        <v>870</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B12" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C12" t="n">
         <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F12" t="n">
-        <v>20</v>
-      </c>
-      <c r="G12" t="n">
-        <v>14</v>
-      </c>
-      <c r="H12" t="n">
-        <v>67</v>
-      </c>
-      <c r="I12" t="n">
-        <v>17</v>
-      </c>
-      <c r="J12" t="n">
         <v>137</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B13" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C13" t="n">
         <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="F13" t="n">
-        <v>22</v>
-      </c>
-      <c r="G13" t="n">
-        <v>15</v>
-      </c>
-      <c r="H13" t="n">
-        <v>45</v>
-      </c>
-      <c r="I13" t="n">
-        <v>18</v>
-      </c>
-      <c r="J13" t="n">
-        <v>870</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B14" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D14" t="n">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="E14" t="n">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="F14" t="n">
-        <v>27</v>
-      </c>
-      <c r="G14" t="n">
-        <v>17</v>
-      </c>
-      <c r="H14" t="n">
-        <v>44</v>
-      </c>
-      <c r="I14" t="n">
-        <v>16</v>
-      </c>
-      <c r="J14" t="n">
-        <v>278</v>
+        <v>252</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B15" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D15" t="n">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="E15" t="n">
         <v>5</v>
       </c>
       <c r="F15" t="n">
-        <v>11</v>
-      </c>
-      <c r="G15" t="n">
-        <v>12</v>
-      </c>
-      <c r="H15" t="n">
-        <v>44</v>
-      </c>
-      <c r="I15" t="n">
-        <v>8</v>
-      </c>
-      <c r="J15" t="n">
-        <v>220</v>
+        <v>144</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" t="n">
         <v>24</v>
       </c>
-      <c r="B16" t="n">
-        <v>20</v>
-      </c>
       <c r="C16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D16" t="n">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="E16" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F16" t="n">
-        <v>12</v>
-      </c>
-      <c r="G16" t="n">
-        <v>7</v>
-      </c>
-      <c r="H16" t="n">
-        <v>59</v>
-      </c>
-      <c r="I16" t="n">
-        <v>5</v>
-      </c>
-      <c r="J16" t="n">
-        <v>144</v>
+        <v>220</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B17" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C17" t="n">
         <v>7</v>
       </c>
       <c r="D17" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E17" t="n">
         <v>8</v>
       </c>
       <c r="F17" t="n">
-        <v>11</v>
-      </c>
-      <c r="G17" t="n">
-        <v>8</v>
-      </c>
-      <c r="H17" t="n">
-        <v>65</v>
-      </c>
-      <c r="I17" t="n">
-        <v>8</v>
-      </c>
-      <c r="J17" t="n">
         <v>171</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B18" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C18" t="n">
         <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="E18" t="n">
         <v>10</v>
       </c>
       <c r="F18" t="n">
-        <v>9</v>
-      </c>
-      <c r="G18" t="n">
-        <v>6</v>
-      </c>
-      <c r="H18" t="n">
-        <v>59</v>
-      </c>
-      <c r="I18" t="n">
-        <v>10</v>
-      </c>
-      <c r="J18" t="n">
         <v>353</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B19" t="n">
         <v>13</v>
       </c>
       <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="n">
         <v>5</v>
       </c>
-      <c r="D19" t="n">
-        <v>8</v>
-      </c>
-      <c r="E19" t="n">
-        <v>17</v>
-      </c>
       <c r="F19" t="n">
-        <v>4</v>
-      </c>
-      <c r="G19" t="n">
-        <v>18</v>
-      </c>
-      <c r="H19" t="n">
-        <v>20</v>
-      </c>
-      <c r="I19" t="n">
-        <v>21</v>
-      </c>
-      <c r="J19" t="n">
-        <v>262</v>
+        <v>167</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B20" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D20" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="E20" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="F20" t="n">
-        <v>3</v>
-      </c>
-      <c r="G20" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" t="n">
-        <v>54</v>
-      </c>
-      <c r="I20" t="n">
-        <v>5</v>
-      </c>
-      <c r="J20" t="n">
-        <v>167</v>
+        <v>262</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B21" t="n">
         <v>11</v>
@@ -1081,24 +829,12 @@
         <v>5</v>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E21" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F21" t="n">
-        <v>6</v>
-      </c>
-      <c r="G21" t="n">
-        <v>16</v>
-      </c>
-      <c r="H21" t="n">
-        <v>2</v>
-      </c>
-      <c r="I21" t="n">
-        <v>23</v>
-      </c>
-      <c r="J21" t="n">
         <v>438</v>
       </c>
     </row>

</xml_diff>

<commit_message>
show all species categories in score tables + add metric labels
</commit_message>
<xml_diff>
--- a/figs/msens-summary_programareas_v3/table_programarea_scores_v3.xlsx
+++ b/figs/msens-summary_programareas_v3/table_programarea_scores_v3.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t xml:space="preserve">Program Area</t>
   </si>
@@ -20,13 +20,28 @@
     <t xml:space="preserve">Score</t>
   </si>
   <si>
+    <t xml:space="preserve">Bird</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invertebrate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mammal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Turtle</t>
+  </si>
+  <si>
     <t xml:space="preserve">Primary Production</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other</t>
   </si>
   <si>
     <t xml:space="preserve">Area (1,000 km2)</t>
@@ -437,370 +452,645 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B2" t="n">
         <v>53</v>
       </c>
       <c r="C2" t="n">
+        <v>39</v>
+      </c>
+      <c r="D2" t="n">
+        <v>48</v>
+      </c>
+      <c r="E2" t="n">
+        <v>70</v>
+      </c>
+      <c r="F2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G2" t="n">
+        <v>84</v>
+      </c>
+      <c r="H2" t="n">
+        <v>33</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2" t="n">
         <v>27</v>
       </c>
-      <c r="D2" t="n">
-        <v>70</v>
-      </c>
-      <c r="E2" t="n">
-        <v>33</v>
-      </c>
-      <c r="F2" t="n">
+      <c r="K2" t="n">
         <v>52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
         <v>48</v>
       </c>
       <c r="C3" t="n">
+        <v>99</v>
+      </c>
+      <c r="D3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E3" t="n">
+        <v>70</v>
+      </c>
+      <c r="F3" t="n">
+        <v>44</v>
+      </c>
+      <c r="G3" t="n">
+        <v>69</v>
+      </c>
+      <c r="H3" t="n">
+        <v>41</v>
+      </c>
+      <c r="I3" t="n">
+        <v>14</v>
+      </c>
+      <c r="J3" t="n">
         <v>21</v>
       </c>
-      <c r="D3" t="n">
-        <v>70</v>
-      </c>
-      <c r="E3" t="n">
-        <v>41</v>
-      </c>
-      <c r="F3" t="n">
+      <c r="K3" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B4" t="n">
         <v>38</v>
       </c>
       <c r="C4" t="n">
+        <v>73</v>
+      </c>
+      <c r="D4" t="n">
+        <v>22</v>
+      </c>
+      <c r="E4" t="n">
+        <v>28</v>
+      </c>
+      <c r="F4" t="n">
+        <v>27</v>
+      </c>
+      <c r="G4" t="n">
+        <v>64</v>
+      </c>
+      <c r="H4" t="n">
+        <v>23</v>
+      </c>
+      <c r="I4" t="n">
+        <v>57</v>
+      </c>
+      <c r="J4" t="n">
         <v>10</v>
       </c>
-      <c r="D4" t="n">
-        <v>28</v>
-      </c>
-      <c r="E4" t="n">
-        <v>23</v>
-      </c>
-      <c r="F4" t="n">
+      <c r="K4" t="n">
         <v>383</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B5" t="n">
         <v>34</v>
       </c>
       <c r="C5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D5" t="n">
+        <v>27</v>
+      </c>
+      <c r="E5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F5" t="n">
+        <v>32</v>
+      </c>
+      <c r="G5" t="n">
+        <v>73</v>
+      </c>
+      <c r="H5" t="n">
+        <v>31</v>
+      </c>
+      <c r="I5" t="n">
         <v>4</v>
       </c>
-      <c r="D5" t="n">
-        <v>37</v>
-      </c>
-      <c r="E5" t="n">
-        <v>31</v>
-      </c>
-      <c r="F5" t="n">
+      <c r="J5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" t="n">
         <v>283</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B6" t="n">
         <v>33</v>
       </c>
       <c r="C6" t="n">
+        <v>59</v>
+      </c>
+      <c r="D6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E6" t="n">
+        <v>31</v>
+      </c>
+      <c r="F6" t="n">
+        <v>32</v>
+      </c>
+      <c r="G6" t="n">
+        <v>40</v>
+      </c>
+      <c r="H6" t="n">
+        <v>26</v>
+      </c>
+      <c r="I6" t="n">
+        <v>54</v>
+      </c>
+      <c r="J6" t="n">
         <v>11</v>
       </c>
-      <c r="D6" t="n">
-        <v>31</v>
-      </c>
-      <c r="E6" t="n">
-        <v>26</v>
-      </c>
-      <c r="F6" t="n">
+      <c r="K6" t="n">
         <v>382</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B7" t="n">
         <v>31</v>
       </c>
       <c r="C7" t="n">
+        <v>74</v>
+      </c>
+      <c r="D7" t="n">
+        <v>14</v>
+      </c>
+      <c r="E7" t="n">
+        <v>26</v>
+      </c>
+      <c r="F7" t="n">
+        <v>19</v>
+      </c>
+      <c r="G7" t="n">
+        <v>47</v>
+      </c>
+      <c r="H7" t="n">
+        <v>17</v>
+      </c>
+      <c r="I7" t="n">
+        <v>41</v>
+      </c>
+      <c r="J7" t="n">
         <v>8</v>
       </c>
-      <c r="D7" t="n">
-        <v>26</v>
-      </c>
-      <c r="E7" t="n">
-        <v>17</v>
-      </c>
-      <c r="F7" t="n">
+      <c r="K7" t="n">
         <v>274</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B8" t="n">
         <v>29</v>
       </c>
       <c r="C8" t="n">
+        <v>63</v>
+      </c>
+      <c r="D8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" t="n">
+        <v>24</v>
+      </c>
+      <c r="F8" t="n">
+        <v>18</v>
+      </c>
+      <c r="G8" t="n">
+        <v>64</v>
+      </c>
+      <c r="H8" t="n">
+        <v>15</v>
+      </c>
+      <c r="I8" t="n">
+        <v>25</v>
+      </c>
+      <c r="J8" t="n">
         <v>10</v>
       </c>
-      <c r="D8" t="n">
-        <v>24</v>
-      </c>
-      <c r="E8" t="n">
-        <v>15</v>
-      </c>
-      <c r="F8" t="n">
+      <c r="K8" t="n">
         <v>276</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B9" t="n">
         <v>28</v>
       </c>
       <c r="C9" t="n">
+        <v>92</v>
+      </c>
+      <c r="D9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" t="n">
+        <v>12</v>
+      </c>
+      <c r="F9" t="n">
+        <v>12</v>
+      </c>
+      <c r="G9" t="n">
+        <v>50</v>
+      </c>
+      <c r="H9" t="n">
+        <v>7</v>
+      </c>
+      <c r="I9"/>
+      <c r="J9" t="n">
         <v>20</v>
       </c>
-      <c r="D9" t="n">
-        <v>12</v>
-      </c>
-      <c r="E9" t="n">
-        <v>7</v>
-      </c>
-      <c r="F9" t="n">
+      <c r="K9" t="n">
         <v>98</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B10" t="n">
         <v>28</v>
       </c>
       <c r="C10" t="n">
+        <v>72</v>
+      </c>
+      <c r="D10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F10" t="n">
+        <v>17</v>
+      </c>
+      <c r="G10" t="n">
+        <v>42</v>
+      </c>
+      <c r="H10" t="n">
+        <v>16</v>
+      </c>
+      <c r="I10" t="n">
+        <v>32</v>
+      </c>
+      <c r="J10" t="n">
         <v>5</v>
       </c>
-      <c r="D10" t="n">
-        <v>27</v>
-      </c>
-      <c r="E10" t="n">
-        <v>16</v>
-      </c>
-      <c r="F10" t="n">
+      <c r="K10" t="n">
         <v>278</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B11" t="n">
         <v>27</v>
       </c>
       <c r="C11" t="n">
+        <v>42</v>
+      </c>
+      <c r="D11" t="n">
+        <v>15</v>
+      </c>
+      <c r="E11" t="n">
+        <v>22</v>
+      </c>
+      <c r="F11" t="n">
+        <v>15</v>
+      </c>
+      <c r="G11" t="n">
+        <v>43</v>
+      </c>
+      <c r="H11" t="n">
+        <v>18</v>
+      </c>
+      <c r="I11" t="n">
+        <v>57</v>
+      </c>
+      <c r="J11" t="n">
         <v>2</v>
       </c>
-      <c r="D11" t="n">
-        <v>22</v>
-      </c>
-      <c r="E11" t="n">
-        <v>18</v>
-      </c>
-      <c r="F11" t="n">
+      <c r="K11" t="n">
         <v>870</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B12" t="n">
         <v>27</v>
       </c>
       <c r="C12" t="n">
+        <v>58</v>
+      </c>
+      <c r="D12" t="n">
+        <v>9</v>
+      </c>
+      <c r="E12" t="n">
+        <v>20</v>
+      </c>
+      <c r="F12" t="n">
+        <v>14</v>
+      </c>
+      <c r="G12" t="n">
+        <v>67</v>
+      </c>
+      <c r="H12" t="n">
+        <v>17</v>
+      </c>
+      <c r="I12"/>
+      <c r="J12" t="n">
         <v>3</v>
       </c>
-      <c r="D12" t="n">
-        <v>20</v>
-      </c>
-      <c r="E12" t="n">
-        <v>17</v>
-      </c>
-      <c r="F12" t="n">
+      <c r="K12" t="n">
         <v>137</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B13" t="n">
         <v>25</v>
       </c>
       <c r="C13" t="n">
+        <v>86</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>14</v>
+      </c>
+      <c r="F13" t="n">
+        <v>12</v>
+      </c>
+      <c r="G13" t="n">
+        <v>55</v>
+      </c>
+      <c r="H13" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" t="n">
+        <v>26</v>
+      </c>
+      <c r="J13" t="n">
         <v>2</v>
       </c>
-      <c r="D13" t="n">
-        <v>14</v>
-      </c>
-      <c r="E13" t="n">
-        <v>6</v>
-      </c>
-      <c r="F13" t="n">
+      <c r="K13" t="n">
         <v>82</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B14" t="n">
         <v>25</v>
       </c>
       <c r="C14" t="n">
+        <v>11</v>
+      </c>
+      <c r="D14" t="n">
+        <v>15</v>
+      </c>
+      <c r="E14" t="n">
+        <v>17</v>
+      </c>
+      <c r="F14" t="n">
+        <v>46</v>
+      </c>
+      <c r="G14" t="n">
+        <v>45</v>
+      </c>
+      <c r="H14" t="n">
+        <v>34</v>
+      </c>
+      <c r="I14"/>
+      <c r="J14" t="n">
         <v>7</v>
       </c>
-      <c r="D14" t="n">
-        <v>17</v>
-      </c>
-      <c r="E14" t="n">
-        <v>34</v>
-      </c>
-      <c r="F14" t="n">
+      <c r="K14" t="n">
         <v>252</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B15" t="n">
         <v>24</v>
       </c>
       <c r="C15" t="n">
+        <v>60</v>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="n">
         <v>12</v>
       </c>
-      <c r="D15" t="n">
+      <c r="F15" t="n">
+        <v>7</v>
+      </c>
+      <c r="G15" t="n">
+        <v>54</v>
+      </c>
+      <c r="H15" t="n">
+        <v>5</v>
+      </c>
+      <c r="I15" t="n">
+        <v>39</v>
+      </c>
+      <c r="J15" t="n">
         <v>12</v>
       </c>
-      <c r="E15" t="n">
-        <v>5</v>
-      </c>
-      <c r="F15" t="n">
+      <c r="K15" t="n">
         <v>144</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B16" t="n">
         <v>24</v>
       </c>
       <c r="C16" t="n">
+        <v>79</v>
+      </c>
+      <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="n">
+        <v>11</v>
+      </c>
+      <c r="F16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G16" t="n">
+        <v>44</v>
+      </c>
+      <c r="H16" t="n">
+        <v>8</v>
+      </c>
+      <c r="I16"/>
+      <c r="J16" t="n">
         <v>10</v>
       </c>
-      <c r="D16" t="n">
-        <v>11</v>
-      </c>
-      <c r="E16" t="n">
-        <v>8</v>
-      </c>
-      <c r="F16" t="n">
+      <c r="K16" t="n">
         <v>220</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B17" t="n">
         <v>23</v>
       </c>
       <c r="C17" t="n">
+        <v>48</v>
+      </c>
+      <c r="D17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E17" t="n">
+        <v>11</v>
+      </c>
+      <c r="F17" t="n">
+        <v>8</v>
+      </c>
+      <c r="G17" t="n">
+        <v>61</v>
+      </c>
+      <c r="H17" t="n">
+        <v>8</v>
+      </c>
+      <c r="I17" t="n">
+        <v>36</v>
+      </c>
+      <c r="J17" t="n">
         <v>7</v>
       </c>
-      <c r="D17" t="n">
-        <v>11</v>
-      </c>
-      <c r="E17" t="n">
-        <v>8</v>
-      </c>
-      <c r="F17" t="n">
+      <c r="K17" t="n">
         <v>171</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B18" t="n">
         <v>19</v>
       </c>
       <c r="C18" t="n">
+        <v>37</v>
+      </c>
+      <c r="D18" t="n">
+        <v>10</v>
+      </c>
+      <c r="E18" t="n">
+        <v>9</v>
+      </c>
+      <c r="F18" t="n">
+        <v>6</v>
+      </c>
+      <c r="G18" t="n">
+        <v>58</v>
+      </c>
+      <c r="H18" t="n">
+        <v>10</v>
+      </c>
+      <c r="I18" t="n">
+        <v>21</v>
+      </c>
+      <c r="J18" t="n">
         <v>2</v>
       </c>
-      <c r="D18" t="n">
-        <v>9</v>
-      </c>
-      <c r="E18" t="n">
-        <v>10</v>
-      </c>
-      <c r="F18" t="n">
+      <c r="K18" t="n">
         <v>353</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B19" t="n">
         <v>13</v>
       </c>
       <c r="C19" t="n">
+        <v>16</v>
+      </c>
+      <c r="D19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="n">
+        <v>53</v>
+      </c>
+      <c r="H19" t="n">
+        <v>5</v>
+      </c>
+      <c r="I19" t="n">
+        <v>20</v>
+      </c>
+      <c r="J19" t="n">
         <v>2</v>
       </c>
-      <c r="D19" t="n">
-        <v>3</v>
-      </c>
-      <c r="E19" t="n">
-        <v>5</v>
-      </c>
-      <c r="F19" t="n">
+      <c r="K19" t="n">
         <v>167</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B20" t="n">
         <v>13</v>
@@ -809,32 +1099,58 @@
         <v>5</v>
       </c>
       <c r="D20" t="n">
+        <v>17</v>
+      </c>
+      <c r="E20" t="n">
         <v>4</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
+        <v>18</v>
+      </c>
+      <c r="G20" t="n">
+        <v>20</v>
+      </c>
+      <c r="H20" t="n">
         <v>21</v>
       </c>
-      <c r="F20" t="n">
+      <c r="I20"/>
+      <c r="J20" t="n">
+        <v>5</v>
+      </c>
+      <c r="K20" t="n">
         <v>262</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B21" t="n">
         <v>11</v>
       </c>
       <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>21</v>
+      </c>
+      <c r="E21" t="n">
+        <v>6</v>
+      </c>
+      <c r="F21" t="n">
+        <v>16</v>
+      </c>
+      <c r="G21" t="n">
+        <v>7</v>
+      </c>
+      <c r="H21" t="n">
+        <v>23</v>
+      </c>
+      <c r="I21"/>
+      <c r="J21" t="n">
         <v>5</v>
       </c>
-      <c r="D21" t="n">
-        <v>6</v>
-      </c>
-      <c r="E21" t="n">
-        <v>23</v>
-      </c>
-      <c r="F21" t="n">
+      <c r="K21" t="n">
         <v>438</v>
       </c>
     </row>

</xml_diff>